<commit_message>
Parser now tracks DQs
</commit_message>
<xml_diff>
--- a/parser/output/season 2.xlsx
+++ b/parser/output/season 2.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6676" uniqueCount="668">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6674" uniqueCount="668">
   <si>
     <t>League Name</t>
   </si>
@@ -2628,19 +2628,19 @@
         <v>6</v>
       </c>
       <c r="B2" s="2">
-        <v>46245.74618281137</v>
+        <v>46245.81005192214</v>
       </c>
       <c r="C2">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="D2">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="E2">
         <v>240</v>
       </c>
       <c r="F2" s="1">
-        <v>0.9416666666666667</v>
+        <v>0.9708333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -5855,9 +5855,6 @@
       <c r="E160">
         <v>0</v>
       </c>
-      <c r="F160" t="s">
-        <v>214</v>
-      </c>
     </row>
     <row r="161" spans="1:6">
       <c r="A161">
@@ -6663,9 +6660,6 @@
       <c r="E201">
         <v>0</v>
       </c>
-      <c r="F201" t="s">
-        <v>214</v>
-      </c>
     </row>
     <row r="202" spans="1:6">
       <c r="A202">
@@ -7034,11 +7028,11 @@
       <c r="C220" t="s">
         <v>32</v>
       </c>
+      <c r="D220" t="s">
+        <v>30</v>
+      </c>
       <c r="E220">
         <v>0</v>
-      </c>
-      <c r="F220" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="221" spans="1:6">
@@ -7382,11 +7376,11 @@
       <c r="C238" t="s">
         <v>50</v>
       </c>
+      <c r="D238" t="s">
+        <v>15</v>
+      </c>
       <c r="E238">
         <v>0</v>
-      </c>
-      <c r="F238" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="239" spans="1:6">
@@ -7399,11 +7393,11 @@
       <c r="C239" t="s">
         <v>30</v>
       </c>
+      <c r="D239" t="s">
+        <v>30</v>
+      </c>
       <c r="E239">
         <v>0</v>
-      </c>
-      <c r="F239" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="240" spans="1:6">
@@ -7416,14 +7410,14 @@
       <c r="C240" t="s">
         <v>34</v>
       </c>
+      <c r="D240" t="s">
+        <v>48</v>
+      </c>
       <c r="E240">
         <v>0</v>
       </c>
-      <c r="F240" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6">
+    </row>
+    <row r="241" spans="1:5">
       <c r="A241">
         <v>12</v>
       </c>
@@ -7433,11 +7427,11 @@
       <c r="C241" t="s">
         <v>53</v>
       </c>
+      <c r="D241" t="s">
+        <v>44</v>
+      </c>
       <c r="E241">
         <v>0</v>
-      </c>
-      <c r="F241" t="s">
-        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -70238,13 +70232,13 @@
         <v>4</v>
       </c>
       <c r="D8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="F8">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -70272,19 +70266,19 @@
         <v>650</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E10">
-        <v>-18</v>
+        <v>-23</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -70292,19 +70286,19 @@
         <v>650</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
       <c r="D11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11">
-        <v>-26</v>
+        <v>-324</v>
       </c>
       <c r="F11">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -70455,16 +70449,16 @@
         <v>30</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D19">
         <v>7</v>
       </c>
       <c r="E19">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -70478,13 +70472,13 @@
         <v>3</v>
       </c>
       <c r="D20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20">
-        <v>-24</v>
+        <v>-27</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -70635,16 +70629,16 @@
         <v>15</v>
       </c>
       <c r="C28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28">
         <v>6</v>
       </c>
       <c r="E28">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="F28">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -70695,16 +70689,16 @@
         <v>44</v>
       </c>
       <c r="C31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31">
         <v>9</v>
       </c>
       <c r="E31">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="F31">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -70798,13 +70792,13 @@
         <v>5</v>
       </c>
       <c r="D36">
+        <v>4</v>
+      </c>
+      <c r="E36">
         <v>3</v>
       </c>
-      <c r="E36">
-        <v>6</v>
-      </c>
       <c r="F36">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -70818,13 +70812,13 @@
         <v>5</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E37">
-        <v>-13</v>
+        <v>-19</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -70872,19 +70866,19 @@
         <v>653</v>
       </c>
       <c r="B40" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
       <c r="D40">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E40">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="F40">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -70892,7 +70886,7 @@
         <v>653</v>
       </c>
       <c r="B41" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -70901,7 +70895,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>-24</v>
+        <v>-28</v>
       </c>
       <c r="F41">
         <v>10</v>
@@ -71102,13 +71096,13 @@
         <v>4</v>
       </c>
       <c r="D8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="F8">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -71136,19 +71130,19 @@
         <v>650</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E10">
-        <v>-18</v>
+        <v>-23</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -71156,19 +71150,19 @@
         <v>650</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
       <c r="D11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11">
-        <v>-26</v>
+        <v>-324</v>
       </c>
       <c r="F11">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -71319,16 +71313,16 @@
         <v>30</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D19">
         <v>7</v>
       </c>
       <c r="E19">
-        <v>-10</v>
+        <v>-4</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -71342,13 +71336,13 @@
         <v>3</v>
       </c>
       <c r="D20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E20">
-        <v>-24</v>
+        <v>-27</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -71499,16 +71493,16 @@
         <v>15</v>
       </c>
       <c r="C28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28">
         <v>6</v>
       </c>
       <c r="E28">
-        <v>-15</v>
+        <v>-12</v>
       </c>
       <c r="F28">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -71559,16 +71553,16 @@
         <v>44</v>
       </c>
       <c r="C31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31">
         <v>9</v>
       </c>
       <c r="E31">
-        <v>-22</v>
+        <v>-19</v>
       </c>
       <c r="F31">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -71662,13 +71656,13 @@
         <v>5</v>
       </c>
       <c r="D36">
+        <v>4</v>
+      </c>
+      <c r="E36">
         <v>3</v>
       </c>
-      <c r="E36">
-        <v>6</v>
-      </c>
       <c r="F36">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -71682,13 +71676,13 @@
         <v>5</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E37">
-        <v>-13</v>
+        <v>-19</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -71736,19 +71730,19 @@
         <v>653</v>
       </c>
       <c r="B40" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
       <c r="D40">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E40">
-        <v>-25</v>
+        <v>-24</v>
       </c>
       <c r="F40">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -71756,7 +71750,7 @@
         <v>653</v>
       </c>
       <c r="B41" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -71765,7 +71759,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>-24</v>
+        <v>-28</v>
       </c>
       <c r="F41">
         <v>10</v>

</xml_diff>